<commit_message>
Fix valuation ratios: use actual year-end market prices (FY17-26) + current price for forecast
</commit_message>
<xml_diff>
--- a/United Spirits Excell - 8 Year + Ratios.xlsx
+++ b/United Spirits Excell - 8 Year + Ratios.xlsx
@@ -31,7 +31,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="21">
+  <numFmts count="22">
     <numFmt numFmtId="164" formatCode="0\A"/>
     <numFmt numFmtId="165" formatCode="0\E"/>
     <numFmt numFmtId="166" formatCode="0.0_);\(0.0\)"/>
@@ -53,6 +53,7 @@
     <numFmt numFmtId="182" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="183" formatCode="0.0&quot;x&quot;"/>
     <numFmt numFmtId="184" formatCode="0.00&quot;x&quot;"/>
+    <numFmt numFmtId="185" formatCode="#,##0.0"/>
   </numFmts>
   <fonts count="33">
     <font>
@@ -905,7 +906,7 @@
     <xf numFmtId="0" fontId="11" fillId="5" borderId="0"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="445">
+  <cellXfs count="446">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -1519,6 +1520,7 @@
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="183" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="184" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="185" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="5">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -21498,7 +21500,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:T45"/>
+  <dimension ref="B2:T46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="2" max="2"/>
@@ -23028,75 +23030,75 @@
         </is>
       </c>
       <c r="C33" s="443">
-        <f>C45/PL!C13</f>
+        <f>C46/PL!C13</f>
         <v/>
       </c>
       <c r="D33" s="443">
-        <f>D45/PL!D13</f>
+        <f>D46/PL!D13</f>
         <v/>
       </c>
       <c r="E33" s="443">
-        <f>E45/PL!E13</f>
+        <f>E46/PL!E13</f>
         <v/>
       </c>
       <c r="F33" s="443">
-        <f>F45/PL!F13</f>
+        <f>F46/PL!F13</f>
         <v/>
       </c>
       <c r="G33" s="443">
-        <f>G45/PL!G13</f>
+        <f>G46/PL!G13</f>
         <v/>
       </c>
       <c r="H33" s="443">
-        <f>H45/PL!H13</f>
+        <f>H46/PL!H13</f>
         <v/>
       </c>
       <c r="I33" s="443">
-        <f>I45/PL!I13</f>
+        <f>I46/PL!I13</f>
         <v/>
       </c>
       <c r="J33" s="443">
-        <f>J45/PL!J13</f>
+        <f>J46/PL!J13</f>
         <v/>
       </c>
       <c r="K33" s="443">
-        <f>K45/PL!K13</f>
+        <f>K46/PL!K13</f>
         <v/>
       </c>
       <c r="L33" s="443">
-        <f>L45/PL!L13</f>
+        <f>L46/PL!L13</f>
         <v/>
       </c>
       <c r="M33" s="443">
-        <f>M45/PL!M13</f>
+        <f>M46/PL!M13</f>
         <v/>
       </c>
       <c r="N33" s="443">
-        <f>N45/PL!N13</f>
+        <f>N46/PL!N13</f>
         <v/>
       </c>
       <c r="O33" s="443">
-        <f>O45/PL!O13</f>
+        <f>O46/PL!O13</f>
         <v/>
       </c>
       <c r="P33" s="443">
-        <f>P45/PL!P13</f>
+        <f>P46/PL!P13</f>
         <v/>
       </c>
       <c r="Q33" s="443">
-        <f>Q45/PL!Q13</f>
+        <f>Q46/PL!Q13</f>
         <v/>
       </c>
       <c r="R33" s="443">
-        <f>R45/PL!R13</f>
+        <f>R46/PL!R13</f>
         <v/>
       </c>
       <c r="S33" s="443">
-        <f>S45/PL!S13</f>
+        <f>S46/PL!S13</f>
         <v/>
       </c>
       <c r="T33" s="443">
-        <f>T45/PL!T13</f>
+        <f>T46/PL!T13</f>
         <v/>
       </c>
     </row>
@@ -23107,75 +23109,75 @@
         </is>
       </c>
       <c r="C34" s="443">
-        <f>C45/PL!C6</f>
+        <f>C46/PL!C6</f>
         <v/>
       </c>
       <c r="D34" s="443">
-        <f>D45/PL!D6</f>
+        <f>D46/PL!D6</f>
         <v/>
       </c>
       <c r="E34" s="443">
-        <f>E45/PL!E6</f>
+        <f>E46/PL!E6</f>
         <v/>
       </c>
       <c r="F34" s="443">
-        <f>F45/PL!F6</f>
+        <f>F46/PL!F6</f>
         <v/>
       </c>
       <c r="G34" s="443">
-        <f>G45/PL!G6</f>
+        <f>G46/PL!G6</f>
         <v/>
       </c>
       <c r="H34" s="443">
-        <f>H45/PL!H6</f>
+        <f>H46/PL!H6</f>
         <v/>
       </c>
       <c r="I34" s="443">
-        <f>I45/PL!I6</f>
+        <f>I46/PL!I6</f>
         <v/>
       </c>
       <c r="J34" s="443">
-        <f>J45/PL!J6</f>
+        <f>J46/PL!J6</f>
         <v/>
       </c>
       <c r="K34" s="443">
-        <f>K45/PL!K6</f>
+        <f>K46/PL!K6</f>
         <v/>
       </c>
       <c r="L34" s="443">
-        <f>L45/PL!L6</f>
+        <f>L46/PL!L6</f>
         <v/>
       </c>
       <c r="M34" s="443">
-        <f>M45/PL!M6</f>
+        <f>M46/PL!M6</f>
         <v/>
       </c>
       <c r="N34" s="443">
-        <f>N45/PL!N6</f>
+        <f>N46/PL!N6</f>
         <v/>
       </c>
       <c r="O34" s="443">
-        <f>O45/PL!O6</f>
+        <f>O46/PL!O6</f>
         <v/>
       </c>
       <c r="P34" s="443">
-        <f>P45/PL!P6</f>
+        <f>P46/PL!P6</f>
         <v/>
       </c>
       <c r="Q34" s="443">
-        <f>Q45/PL!Q6</f>
+        <f>Q46/PL!Q6</f>
         <v/>
       </c>
       <c r="R34" s="443">
-        <f>R45/PL!R6</f>
+        <f>R46/PL!R6</f>
         <v/>
       </c>
       <c r="S34" s="443">
-        <f>S45/PL!S6</f>
+        <f>S46/PL!S6</f>
         <v/>
       </c>
       <c r="T34" s="443">
-        <f>T45/PL!T6</f>
+        <f>T46/PL!T6</f>
         <v/>
       </c>
     </row>
@@ -23186,75 +23188,75 @@
         </is>
       </c>
       <c r="C35" s="443">
-        <f>C45/PL!C15</f>
+        <f>C46/PL!C15</f>
         <v/>
       </c>
       <c r="D35" s="443">
-        <f>D45/PL!D15</f>
+        <f>D46/PL!D15</f>
         <v/>
       </c>
       <c r="E35" s="443">
-        <f>E45/PL!E15</f>
+        <f>E46/PL!E15</f>
         <v/>
       </c>
       <c r="F35" s="443">
-        <f>F45/PL!F15</f>
+        <f>F46/PL!F15</f>
         <v/>
       </c>
       <c r="G35" s="443">
-        <f>G45/PL!G15</f>
+        <f>G46/PL!G15</f>
         <v/>
       </c>
       <c r="H35" s="443">
-        <f>H45/PL!H15</f>
+        <f>H46/PL!H15</f>
         <v/>
       </c>
       <c r="I35" s="443">
-        <f>I45/PL!I15</f>
+        <f>I46/PL!I15</f>
         <v/>
       </c>
       <c r="J35" s="443">
-        <f>J45/PL!J15</f>
+        <f>J46/PL!J15</f>
         <v/>
       </c>
       <c r="K35" s="443">
-        <f>K45/PL!K15</f>
+        <f>K46/PL!K15</f>
         <v/>
       </c>
       <c r="L35" s="443">
-        <f>L45/PL!L15</f>
+        <f>L46/PL!L15</f>
         <v/>
       </c>
       <c r="M35" s="443">
-        <f>M45/PL!M15</f>
+        <f>M46/PL!M15</f>
         <v/>
       </c>
       <c r="N35" s="443">
-        <f>N45/PL!N15</f>
+        <f>N46/PL!N15</f>
         <v/>
       </c>
       <c r="O35" s="443">
-        <f>O45/PL!O15</f>
+        <f>O46/PL!O15</f>
         <v/>
       </c>
       <c r="P35" s="443">
-        <f>P45/PL!P15</f>
+        <f>P46/PL!P15</f>
         <v/>
       </c>
       <c r="Q35" s="443">
-        <f>Q45/PL!Q15</f>
+        <f>Q46/PL!Q15</f>
         <v/>
       </c>
       <c r="R35" s="443">
-        <f>R45/PL!R15</f>
+        <f>R46/PL!R15</f>
         <v/>
       </c>
       <c r="S35" s="443">
-        <f>S45/PL!S15</f>
+        <f>S46/PL!S15</f>
         <v/>
       </c>
       <c r="T35" s="443">
-        <f>T45/PL!T15</f>
+        <f>T46/PL!T15</f>
         <v/>
       </c>
     </row>
@@ -23265,82 +23267,82 @@
         </is>
       </c>
       <c r="C36" s="443">
-        <f>C41/PL!C23</f>
+        <f>C42/PL!C23</f>
         <v/>
       </c>
       <c r="D36" s="443">
-        <f>D41/PL!D23</f>
+        <f>D42/PL!D23</f>
         <v/>
       </c>
       <c r="E36" s="443">
-        <f>E41/PL!E23</f>
+        <f>E42/PL!E23</f>
         <v/>
       </c>
       <c r="F36" s="443">
-        <f>F41/PL!F23</f>
+        <f>F42/PL!F23</f>
         <v/>
       </c>
       <c r="G36" s="443">
-        <f>G41/PL!G23</f>
+        <f>G42/PL!G23</f>
         <v/>
       </c>
       <c r="H36" s="443">
-        <f>H41/PL!H23</f>
+        <f>H42/PL!H23</f>
         <v/>
       </c>
       <c r="I36" s="443">
-        <f>I41/PL!I23</f>
+        <f>I42/PL!I23</f>
         <v/>
       </c>
       <c r="J36" s="443">
-        <f>J41/PL!J23</f>
+        <f>J42/PL!J23</f>
         <v/>
       </c>
       <c r="K36" s="443">
-        <f>K41/PL!K23</f>
+        <f>K42/PL!K23</f>
         <v/>
       </c>
       <c r="L36" s="443">
-        <f>L41/PL!L23</f>
+        <f>L42/PL!L23</f>
         <v/>
       </c>
       <c r="M36" s="443">
-        <f>M41/PL!M23</f>
+        <f>M42/PL!M23</f>
         <v/>
       </c>
       <c r="N36" s="443">
-        <f>N41/PL!N23</f>
+        <f>N42/PL!N23</f>
         <v/>
       </c>
       <c r="O36" s="443">
-        <f>O41/PL!O23</f>
+        <f>O42/PL!O23</f>
         <v/>
       </c>
       <c r="P36" s="443">
-        <f>P41/PL!P23</f>
+        <f>P42/PL!P23</f>
         <v/>
       </c>
       <c r="Q36" s="443">
-        <f>Q41/PL!Q23</f>
+        <f>Q42/PL!Q23</f>
         <v/>
       </c>
       <c r="R36" s="443">
-        <f>R41/PL!R23</f>
+        <f>R42/PL!R23</f>
         <v/>
       </c>
       <c r="S36" s="443">
-        <f>S41/PL!S23</f>
+        <f>S42/PL!S23</f>
         <v/>
       </c>
       <c r="T36" s="443">
-        <f>T41/PL!T23</f>
+        <f>T42/PL!T23</f>
         <v/>
       </c>
     </row>
     <row r="39">
       <c r="B39" s="441" t="inlineStr">
         <is>
-          <t>Memo - valuation basis (Market Cap held at current level)</t>
+          <t>Memo - valuation basis  (actual year-end market price; FY27-34 held at current price Rs1,246.7)</t>
         </is>
       </c>
       <c r="C39" s="442" t="n"/>
@@ -23362,398 +23364,520 @@
       <c r="S39" s="442" t="n"/>
       <c r="T39" s="442" t="n"/>
     </row>
+    <row r="40">
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Year-end Share Price (Rs)</t>
+        </is>
+      </c>
+      <c r="C40" s="445" t="n">
+        <v>434.3</v>
+      </c>
+      <c r="D40" s="445" t="n">
+        <v>624.5</v>
+      </c>
+      <c r="E40" s="445" t="n">
+        <v>539.5</v>
+      </c>
+      <c r="F40" s="445" t="n">
+        <v>490</v>
+      </c>
+      <c r="G40" s="445" t="n">
+        <v>519.5</v>
+      </c>
+      <c r="H40" s="445" t="n">
+        <v>862.9</v>
+      </c>
+      <c r="I40" s="445" t="n">
+        <v>777.1</v>
+      </c>
+      <c r="J40" s="445" t="n">
+        <v>1128.3</v>
+      </c>
+      <c r="K40" s="445" t="n">
+        <v>1427.3</v>
+      </c>
+      <c r="L40" s="445" t="n">
+        <v>1325.6</v>
+      </c>
+      <c r="M40" s="445" t="n">
+        <v>1246.7</v>
+      </c>
+      <c r="N40" s="445" t="n">
+        <v>1246.7</v>
+      </c>
+      <c r="O40" s="445" t="n">
+        <v>1246.7</v>
+      </c>
+      <c r="P40" s="445" t="n">
+        <v>1246.7</v>
+      </c>
+      <c r="Q40" s="445" t="n">
+        <v>1246.7</v>
+      </c>
+      <c r="R40" s="445" t="n">
+        <v>1246.7</v>
+      </c>
+      <c r="S40" s="445" t="n">
+        <v>1246.7</v>
+      </c>
+      <c r="T40" s="445" t="n">
+        <v>1246.7</v>
+      </c>
+    </row>
     <row r="41">
       <c r="B41" t="inlineStr">
         <is>
-          <t>Market Cap (current, constant)</t>
-        </is>
-      </c>
-      <c r="C41" s="1">
-        <f>Comparables!$C$12</f>
-        <v/>
-      </c>
-      <c r="D41" s="1">
-        <f>Comparables!$C$12</f>
-        <v/>
-      </c>
-      <c r="E41" s="1">
-        <f>Comparables!$C$12</f>
-        <v/>
-      </c>
-      <c r="F41" s="1">
-        <f>Comparables!$C$12</f>
-        <v/>
-      </c>
-      <c r="G41" s="1">
-        <f>Comparables!$C$12</f>
-        <v/>
-      </c>
-      <c r="H41" s="1">
-        <f>Comparables!$C$12</f>
-        <v/>
-      </c>
-      <c r="I41" s="1">
-        <f>Comparables!$C$12</f>
-        <v/>
-      </c>
-      <c r="J41" s="1">
-        <f>Comparables!$C$12</f>
-        <v/>
-      </c>
-      <c r="K41" s="1">
-        <f>Comparables!$C$12</f>
-        <v/>
-      </c>
-      <c r="L41" s="1">
-        <f>Comparables!$C$12</f>
-        <v/>
-      </c>
-      <c r="M41" s="1">
-        <f>Comparables!$C$12</f>
-        <v/>
-      </c>
-      <c r="N41" s="1">
-        <f>Comparables!$C$12</f>
-        <v/>
-      </c>
-      <c r="O41" s="1">
-        <f>Comparables!$C$12</f>
-        <v/>
-      </c>
-      <c r="P41" s="1">
-        <f>Comparables!$C$12</f>
-        <v/>
-      </c>
-      <c r="Q41" s="1">
-        <f>Comparables!$C$12</f>
-        <v/>
-      </c>
-      <c r="R41" s="1">
-        <f>Comparables!$C$12</f>
-        <v/>
-      </c>
-      <c r="S41" s="1">
-        <f>Comparables!$C$12</f>
-        <v/>
-      </c>
-      <c r="T41" s="1">
-        <f>Comparables!$C$12</f>
-        <v/>
+          <t>Shares Outstanding (cr)</t>
+        </is>
+      </c>
+      <c r="C41" s="15" t="n">
+        <v>72.73999999999999</v>
+      </c>
+      <c r="D41" s="15" t="n">
+        <v>72.73999999999999</v>
+      </c>
+      <c r="E41" s="15" t="n">
+        <v>72.73999999999999</v>
+      </c>
+      <c r="F41" s="15" t="n">
+        <v>72.73999999999999</v>
+      </c>
+      <c r="G41" s="15" t="n">
+        <v>72.73999999999999</v>
+      </c>
+      <c r="H41" s="15" t="n">
+        <v>72.73999999999999</v>
+      </c>
+      <c r="I41" s="15" t="n">
+        <v>72.73999999999999</v>
+      </c>
+      <c r="J41" s="15" t="n">
+        <v>72.73999999999999</v>
+      </c>
+      <c r="K41" s="15" t="n">
+        <v>72.73999999999999</v>
+      </c>
+      <c r="L41" s="15" t="n">
+        <v>72.73999999999999</v>
+      </c>
+      <c r="M41" s="15" t="n">
+        <v>72.73999999999999</v>
+      </c>
+      <c r="N41" s="15" t="n">
+        <v>72.73999999999999</v>
+      </c>
+      <c r="O41" s="15" t="n">
+        <v>72.73999999999999</v>
+      </c>
+      <c r="P41" s="15" t="n">
+        <v>72.73999999999999</v>
+      </c>
+      <c r="Q41" s="15" t="n">
+        <v>72.73999999999999</v>
+      </c>
+      <c r="R41" s="15" t="n">
+        <v>72.73999999999999</v>
+      </c>
+      <c r="S41" s="15" t="n">
+        <v>72.73999999999999</v>
+      </c>
+      <c r="T41" s="15" t="n">
+        <v>72.73999999999999</v>
       </c>
     </row>
     <row r="42">
       <c r="B42" t="inlineStr">
         <is>
-          <t>Total Debt (borrowings + leases)</t>
+          <t>Market Capitalisation (Rs cr)</t>
         </is>
       </c>
       <c r="C42" s="1">
-        <f>BS!C15+BS!C17+BS!C22</f>
+        <f>C40*C41</f>
         <v/>
       </c>
       <c r="D42" s="1">
-        <f>BS!D15+BS!D17+BS!D22</f>
+        <f>D40*D41</f>
         <v/>
       </c>
       <c r="E42" s="1">
-        <f>BS!E15+BS!E17+BS!E22</f>
+        <f>E40*E41</f>
         <v/>
       </c>
       <c r="F42" s="1">
-        <f>BS!F15+BS!F17+BS!F22</f>
+        <f>F40*F41</f>
         <v/>
       </c>
       <c r="G42" s="1">
-        <f>BS!G15+BS!G17+BS!G22</f>
+        <f>G40*G41</f>
         <v/>
       </c>
       <c r="H42" s="1">
-        <f>BS!H15+BS!H17+BS!H22</f>
+        <f>H40*H41</f>
         <v/>
       </c>
       <c r="I42" s="1">
-        <f>BS!I15+BS!I17+BS!I22</f>
+        <f>I40*I41</f>
         <v/>
       </c>
       <c r="J42" s="1">
-        <f>BS!J15+BS!J17+BS!J22</f>
+        <f>J40*J41</f>
         <v/>
       </c>
       <c r="K42" s="1">
-        <f>BS!K15+BS!K17+BS!K22</f>
+        <f>K40*K41</f>
         <v/>
       </c>
       <c r="L42" s="1">
-        <f>BS!L15+BS!L17+BS!L22</f>
+        <f>L40*L41</f>
         <v/>
       </c>
       <c r="M42" s="1">
-        <f>BS!M15+BS!M17+BS!M22</f>
+        <f>M40*M41</f>
         <v/>
       </c>
       <c r="N42" s="1">
-        <f>BS!N15+BS!N17+BS!N22</f>
+        <f>N40*N41</f>
         <v/>
       </c>
       <c r="O42" s="1">
-        <f>BS!O15+BS!O17+BS!O22</f>
+        <f>O40*O41</f>
         <v/>
       </c>
       <c r="P42" s="1">
-        <f>BS!P15+BS!P17+BS!P22</f>
+        <f>P40*P41</f>
         <v/>
       </c>
       <c r="Q42" s="1">
-        <f>BS!Q15+BS!Q17+BS!Q22</f>
+        <f>Q40*Q41</f>
         <v/>
       </c>
       <c r="R42" s="1">
-        <f>BS!R15+BS!R17+BS!R22</f>
+        <f>R40*R41</f>
         <v/>
       </c>
       <c r="S42" s="1">
-        <f>BS!S15+BS!S17+BS!S22</f>
+        <f>S40*S41</f>
         <v/>
       </c>
       <c r="T42" s="1">
-        <f>BS!T15+BS!T17+BS!T22</f>
+        <f>T40*T41</f>
         <v/>
       </c>
     </row>
     <row r="43">
       <c r="B43" t="inlineStr">
         <is>
-          <t>Cash &amp; Investments</t>
+          <t>Total Debt (borrowings + leases)</t>
         </is>
       </c>
       <c r="C43" s="1">
-        <f>BS!C45</f>
+        <f>BS!C15+BS!C17+BS!C22</f>
         <v/>
       </c>
       <c r="D43" s="1">
-        <f>BS!D45</f>
+        <f>BS!D15+BS!D17+BS!D22</f>
         <v/>
       </c>
       <c r="E43" s="1">
-        <f>BS!E45</f>
+        <f>BS!E15+BS!E17+BS!E22</f>
         <v/>
       </c>
       <c r="F43" s="1">
-        <f>BS!F45</f>
+        <f>BS!F15+BS!F17+BS!F22</f>
         <v/>
       </c>
       <c r="G43" s="1">
-        <f>BS!G45</f>
+        <f>BS!G15+BS!G17+BS!G22</f>
         <v/>
       </c>
       <c r="H43" s="1">
-        <f>BS!H45</f>
+        <f>BS!H15+BS!H17+BS!H22</f>
         <v/>
       </c>
       <c r="I43" s="1">
-        <f>BS!I45</f>
+        <f>BS!I15+BS!I17+BS!I22</f>
         <v/>
       </c>
       <c r="J43" s="1">
-        <f>BS!J45</f>
+        <f>BS!J15+BS!J17+BS!J22</f>
         <v/>
       </c>
       <c r="K43" s="1">
-        <f>BS!K45</f>
+        <f>BS!K15+BS!K17+BS!K22</f>
         <v/>
       </c>
       <c r="L43" s="1">
-        <f>BS!L45</f>
+        <f>BS!L15+BS!L17+BS!L22</f>
         <v/>
       </c>
       <c r="M43" s="1">
-        <f>BS!M45</f>
+        <f>BS!M15+BS!M17+BS!M22</f>
         <v/>
       </c>
       <c r="N43" s="1">
-        <f>BS!N45</f>
+        <f>BS!N15+BS!N17+BS!N22</f>
         <v/>
       </c>
       <c r="O43" s="1">
-        <f>BS!O45</f>
+        <f>BS!O15+BS!O17+BS!O22</f>
         <v/>
       </c>
       <c r="P43" s="1">
-        <f>BS!P45</f>
+        <f>BS!P15+BS!P17+BS!P22</f>
         <v/>
       </c>
       <c r="Q43" s="1">
-        <f>BS!Q45</f>
+        <f>BS!Q15+BS!Q17+BS!Q22</f>
         <v/>
       </c>
       <c r="R43" s="1">
-        <f>BS!R45</f>
+        <f>BS!R15+BS!R17+BS!R22</f>
         <v/>
       </c>
       <c r="S43" s="1">
-        <f>BS!S45</f>
+        <f>BS!S15+BS!S17+BS!S22</f>
         <v/>
       </c>
       <c r="T43" s="1">
-        <f>BS!T45</f>
+        <f>BS!T15+BS!T17+BS!T22</f>
         <v/>
       </c>
     </row>
     <row r="44">
       <c r="B44" t="inlineStr">
         <is>
-          <t>Net Debt</t>
+          <t>Cash &amp; Investments</t>
         </is>
       </c>
       <c r="C44" s="1">
-        <f>C42-C43</f>
+        <f>BS!C45</f>
         <v/>
       </c>
       <c r="D44" s="1">
-        <f>D42-D43</f>
+        <f>BS!D45</f>
         <v/>
       </c>
       <c r="E44" s="1">
-        <f>E42-E43</f>
+        <f>BS!E45</f>
         <v/>
       </c>
       <c r="F44" s="1">
-        <f>F42-F43</f>
+        <f>BS!F45</f>
         <v/>
       </c>
       <c r="G44" s="1">
-        <f>G42-G43</f>
+        <f>BS!G45</f>
         <v/>
       </c>
       <c r="H44" s="1">
-        <f>H42-H43</f>
+        <f>BS!H45</f>
         <v/>
       </c>
       <c r="I44" s="1">
-        <f>I42-I43</f>
+        <f>BS!I45</f>
         <v/>
       </c>
       <c r="J44" s="1">
-        <f>J42-J43</f>
+        <f>BS!J45</f>
         <v/>
       </c>
       <c r="K44" s="1">
-        <f>K42-K43</f>
+        <f>BS!K45</f>
         <v/>
       </c>
       <c r="L44" s="1">
-        <f>L42-L43</f>
+        <f>BS!L45</f>
         <v/>
       </c>
       <c r="M44" s="1">
-        <f>M42-M43</f>
+        <f>BS!M45</f>
         <v/>
       </c>
       <c r="N44" s="1">
-        <f>N42-N43</f>
+        <f>BS!N45</f>
         <v/>
       </c>
       <c r="O44" s="1">
-        <f>O42-O43</f>
+        <f>BS!O45</f>
         <v/>
       </c>
       <c r="P44" s="1">
-        <f>P42-P43</f>
+        <f>BS!P45</f>
         <v/>
       </c>
       <c r="Q44" s="1">
-        <f>Q42-Q43</f>
+        <f>BS!Q45</f>
         <v/>
       </c>
       <c r="R44" s="1">
-        <f>R42-R43</f>
+        <f>BS!R45</f>
         <v/>
       </c>
       <c r="S44" s="1">
-        <f>S42-S43</f>
+        <f>BS!S45</f>
         <v/>
       </c>
       <c r="T44" s="1">
-        <f>T42-T43</f>
+        <f>BS!T45</f>
         <v/>
       </c>
     </row>
     <row r="45">
       <c r="B45" t="inlineStr">
         <is>
+          <t>Net Debt</t>
+        </is>
+      </c>
+      <c r="C45" s="1">
+        <f>C43-C44</f>
+        <v/>
+      </c>
+      <c r="D45" s="1">
+        <f>D43-D44</f>
+        <v/>
+      </c>
+      <c r="E45" s="1">
+        <f>E43-E44</f>
+        <v/>
+      </c>
+      <c r="F45" s="1">
+        <f>F43-F44</f>
+        <v/>
+      </c>
+      <c r="G45" s="1">
+        <f>G43-G44</f>
+        <v/>
+      </c>
+      <c r="H45" s="1">
+        <f>H43-H44</f>
+        <v/>
+      </c>
+      <c r="I45" s="1">
+        <f>I43-I44</f>
+        <v/>
+      </c>
+      <c r="J45" s="1">
+        <f>J43-J44</f>
+        <v/>
+      </c>
+      <c r="K45" s="1">
+        <f>K43-K44</f>
+        <v/>
+      </c>
+      <c r="L45" s="1">
+        <f>L43-L44</f>
+        <v/>
+      </c>
+      <c r="M45" s="1">
+        <f>M43-M44</f>
+        <v/>
+      </c>
+      <c r="N45" s="1">
+        <f>N43-N44</f>
+        <v/>
+      </c>
+      <c r="O45" s="1">
+        <f>O43-O44</f>
+        <v/>
+      </c>
+      <c r="P45" s="1">
+        <f>P43-P44</f>
+        <v/>
+      </c>
+      <c r="Q45" s="1">
+        <f>Q43-Q44</f>
+        <v/>
+      </c>
+      <c r="R45" s="1">
+        <f>R43-R44</f>
+        <v/>
+      </c>
+      <c r="S45" s="1">
+        <f>S43-S44</f>
+        <v/>
+      </c>
+      <c r="T45" s="1">
+        <f>T43-T44</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="B46" t="inlineStr">
+        <is>
           <t>Enterprise Value (Mkt Cap + Net Debt)</t>
         </is>
       </c>
-      <c r="C45" s="1">
-        <f>C41+C44</f>
-        <v/>
-      </c>
-      <c r="D45" s="1">
-        <f>D41+D44</f>
-        <v/>
-      </c>
-      <c r="E45" s="1">
-        <f>E41+E44</f>
-        <v/>
-      </c>
-      <c r="F45" s="1">
-        <f>F41+F44</f>
-        <v/>
-      </c>
-      <c r="G45" s="1">
-        <f>G41+G44</f>
-        <v/>
-      </c>
-      <c r="H45" s="1">
-        <f>H41+H44</f>
-        <v/>
-      </c>
-      <c r="I45" s="1">
-        <f>I41+I44</f>
-        <v/>
-      </c>
-      <c r="J45" s="1">
-        <f>J41+J44</f>
-        <v/>
-      </c>
-      <c r="K45" s="1">
-        <f>K41+K44</f>
-        <v/>
-      </c>
-      <c r="L45" s="1">
-        <f>L41+L44</f>
-        <v/>
-      </c>
-      <c r="M45" s="1">
-        <f>M41+M44</f>
-        <v/>
-      </c>
-      <c r="N45" s="1">
-        <f>N41+N44</f>
-        <v/>
-      </c>
-      <c r="O45" s="1">
-        <f>O41+O44</f>
-        <v/>
-      </c>
-      <c r="P45" s="1">
-        <f>P41+P44</f>
-        <v/>
-      </c>
-      <c r="Q45" s="1">
-        <f>Q41+Q44</f>
-        <v/>
-      </c>
-      <c r="R45" s="1">
-        <f>R41+R44</f>
-        <v/>
-      </c>
-      <c r="S45" s="1">
-        <f>S41+S44</f>
-        <v/>
-      </c>
-      <c r="T45" s="1">
-        <f>T41+T44</f>
+      <c r="C46" s="1">
+        <f>C42+C45</f>
+        <v/>
+      </c>
+      <c r="D46" s="1">
+        <f>D42+D45</f>
+        <v/>
+      </c>
+      <c r="E46" s="1">
+        <f>E42+E45</f>
+        <v/>
+      </c>
+      <c r="F46" s="1">
+        <f>F42+F45</f>
+        <v/>
+      </c>
+      <c r="G46" s="1">
+        <f>G42+G45</f>
+        <v/>
+      </c>
+      <c r="H46" s="1">
+        <f>H42+H45</f>
+        <v/>
+      </c>
+      <c r="I46" s="1">
+        <f>I42+I45</f>
+        <v/>
+      </c>
+      <c r="J46" s="1">
+        <f>J42+J45</f>
+        <v/>
+      </c>
+      <c r="K46" s="1">
+        <f>K42+K45</f>
+        <v/>
+      </c>
+      <c r="L46" s="1">
+        <f>L42+L45</f>
+        <v/>
+      </c>
+      <c r="M46" s="1">
+        <f>M42+M45</f>
+        <v/>
+      </c>
+      <c r="N46" s="1">
+        <f>N42+N45</f>
+        <v/>
+      </c>
+      <c r="O46" s="1">
+        <f>O42+O45</f>
+        <v/>
+      </c>
+      <c r="P46" s="1">
+        <f>P42+P45</f>
+        <v/>
+      </c>
+      <c r="Q46" s="1">
+        <f>Q42+Q45</f>
+        <v/>
+      </c>
+      <c r="R46" s="1">
+        <f>R42+R45</f>
+        <v/>
+      </c>
+      <c r="S46" s="1">
+        <f>S42+S45</f>
+        <v/>
+      </c>
+      <c r="T46" s="1">
+        <f>T42+T45</f>
         <v/>
       </c>
     </row>

</xml_diff>